<commit_message>
fix: correct KC_19 document name from HVAC to Kết cấu and add gitignore
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -20280,7 +20280,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Tài liệu tập hợp các lỗi hay gặp trong thiết kế HVAC các hạng mục</t>
+          <t>Tài liệu tập hợp các lỗi hay gặp trong thiết kế Kết cấu các hạng mục</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Lưu ý: Bản gốc ghi nhầm 'HVAC', cần đổi thành 'Kết cấu'</t>
+          <t>Bình thường</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: replace pending hire position with Nhân sự M
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (BIM Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Khuyết nhân sự chủ chốt</t>
+          <t>Đang làm việc</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Chưa tuyển đủ</t>
+          <t>KS Triển khai HVAC</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -4095,7 +4095,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5967,7 +5967,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -6903,7 +6903,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -11115,7 +11115,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -12519,7 +12519,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -13455,7 +13455,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -13923,7 +13923,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -14391,7 +14391,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -14859,7 +14859,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -15327,7 +15327,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -15795,7 +15795,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -16731,7 +16731,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -17199,7 +17199,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -17667,7 +17667,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Vị trí chờ tuyển (Hạ tầng)</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">

</xml_diff>

<commit_message>
feat: rename project filter and projects to 'Dự án Mẫu' (Dự án Mẫu 01 - 07)
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -678,12 +678,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ty Le Hoan Thanh Du An = DIVIDE(CALCULATE(COUNTROWS('07_Fact_BaoCaoCongViec'), '07_Fact_BaoCaoCongViec'[TinhTrang] = "Đã hoàn thành", '07_Fact_BaoCaoCongViec'[NhomCongViec] = "Dự án Thi công"), CALCULATE(COUNTROWS('07_Fact_BaoCaoCongViec'), '07_Fact_BaoCaoCongViec'[NhomCongViec] = "Dự án Thi công"), 0)</t>
+          <t>Ty Le Hoan Thanh Du An = DIVIDE(CALCULATE(COUNTROWS('07_Fact_BaoCaoCongViec'), '07_Fact_BaoCaoCongViec'[TinhTrang] = "Đã hoàn thành", '07_Fact_BaoCaoCongViec'[NhomCongViec] = "Dự án Mẫu (Thi công &amp; Triển khai)"), CALCULATE(COUNTROWS('07_Fact_BaoCaoCongViec'), '07_Fact_BaoCaoCongViec'[NhomCongViec] = "Dự án Mẫu (Thi công &amp; Triển khai)"), 0)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Gauge Chart tiến độ 7 dự án</t>
+          <t>Gauge Chart tiến độ 7 dự án mẫu</t>
         </is>
       </c>
     </row>
@@ -30715,12 +30715,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -30767,12 +30767,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -30819,12 +30819,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -30871,12 +30871,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -30923,12 +30923,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -30975,12 +30975,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -31027,12 +31027,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -31079,12 +31079,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -31131,12 +31131,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -31183,12 +31183,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31235,12 +31235,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31287,12 +31287,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -31339,12 +31339,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -31391,12 +31391,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -31443,12 +31443,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -31495,12 +31495,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -31547,12 +31547,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -31599,12 +31599,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -31651,12 +31651,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -31703,12 +31703,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -31755,12 +31755,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -31807,12 +31807,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -31859,12 +31859,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -31907,12 +31907,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dự án Mega</t>
+          <t>Dự án Mẫu 01 (Mega)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -31951,12 +31951,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -32003,12 +32003,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -32055,12 +32055,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -32107,12 +32107,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -32159,12 +32159,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -32211,12 +32211,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -32263,12 +32263,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -32315,12 +32315,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -32367,12 +32367,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -32419,12 +32419,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -32471,12 +32471,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -32523,12 +32523,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Dự án CasaFlora2</t>
+          <t>Dự án Mẫu 04 (CasaFlora2)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -32575,12 +32575,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -32627,12 +32627,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -32679,12 +32679,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -32731,12 +32731,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -32783,12 +32783,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -32831,12 +32831,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -32875,12 +32875,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -32927,12 +32927,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -32975,12 +32975,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -33027,12 +33027,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -33079,12 +33079,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -33127,12 +33127,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -33179,12 +33179,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -33231,12 +33231,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -33279,12 +33279,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -33331,12 +33331,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -33379,12 +33379,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -33431,12 +33431,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Dự án Kim Tín giai đoạn 3</t>
+          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -33483,12 +33483,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -33535,12 +33535,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -33587,12 +33587,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -33631,12 +33631,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -33683,12 +33683,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -33735,12 +33735,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -33787,12 +33787,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -33835,12 +33835,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -33879,12 +33879,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -33923,12 +33923,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -33967,12 +33967,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -34011,12 +34011,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -34055,12 +34055,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -34099,12 +34099,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -34143,12 +34143,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Dự án APF</t>
+          <t>Dự án Mẫu 03 (APF)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -34187,12 +34187,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -34239,12 +34239,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -34291,12 +34291,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -34343,12 +34343,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -34395,12 +34395,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -34447,12 +34447,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -34499,12 +34499,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -34551,12 +34551,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -34599,12 +34599,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dự án Suncasa</t>
+          <t>Dự án Mẫu 05 (Suncasa)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -34647,12 +34647,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -34699,12 +34699,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -34751,12 +34751,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -34803,12 +34803,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -34855,12 +34855,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -34907,12 +34907,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -34959,12 +34959,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dự án các trạm Phú Quốc</t>
+          <t>Dự án Mẫu 06 (Phú Quốc)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -35011,12 +35011,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Dự án BB052</t>
+          <t>Dự án Mẫu 07 (BB052)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -35063,12 +35063,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Dự án Thi công</t>
+          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Dự án BB052</t>
+          <t>Dự án Mẫu 07 (BB052)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">

</xml_diff>

<commit_message>
feat: consolidate all project tasks into a single 'Dự án Mẫu' (87 tasks) and streamline filter
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -30720,7 +30720,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -30772,7 +30772,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -30824,7 +30824,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -30876,7 +30876,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -30928,7 +30928,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -30980,7 +30980,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -31032,7 +31032,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -31084,7 +31084,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -31136,7 +31136,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -31188,7 +31188,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31240,7 +31240,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31292,7 +31292,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -31344,7 +31344,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -31396,7 +31396,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -31448,7 +31448,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -31500,7 +31500,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -31552,7 +31552,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -31604,7 +31604,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -31656,7 +31656,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -31708,7 +31708,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -31760,7 +31760,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -31812,7 +31812,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -31864,7 +31864,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -31912,7 +31912,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 01 (Mega)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -31956,7 +31956,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -32008,7 +32008,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -32060,7 +32060,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -32112,7 +32112,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -32164,7 +32164,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -32216,7 +32216,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -32268,7 +32268,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -32320,7 +32320,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -32372,7 +32372,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -32424,7 +32424,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -32476,7 +32476,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -32528,7 +32528,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 04 (CasaFlora2)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -32580,7 +32580,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -32684,7 +32684,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -32736,7 +32736,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -32788,7 +32788,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -32836,7 +32836,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -32880,7 +32880,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -32932,7 +32932,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -32980,7 +32980,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -33032,7 +33032,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -33132,7 +33132,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -33184,7 +33184,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -33236,7 +33236,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -33284,7 +33284,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -33336,7 +33336,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -33436,7 +33436,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 02 (Kim Tín GĐ3)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -33488,7 +33488,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -33540,7 +33540,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -33592,7 +33592,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -33636,7 +33636,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -33688,7 +33688,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -33740,7 +33740,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -33792,7 +33792,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -33884,7 +33884,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -33928,7 +33928,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -33972,7 +33972,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -34016,7 +34016,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -34060,7 +34060,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -34104,7 +34104,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -34148,7 +34148,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 03 (APF)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -34192,7 +34192,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -34244,7 +34244,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -34348,7 +34348,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -34400,7 +34400,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -34452,7 +34452,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -34504,7 +34504,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -34556,7 +34556,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -34604,7 +34604,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 05 (Suncasa)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -34652,7 +34652,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -34704,7 +34704,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -34756,7 +34756,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -34808,7 +34808,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -34860,7 +34860,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -34912,7 +34912,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -34964,7 +34964,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 06 (Phú Quốc)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -35016,7 +35016,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 07 (BB052)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -35068,7 +35068,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Dự án Mẫu 07 (BB052)</t>
+          <t>Dự án Mẫu</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">

</xml_diff>

<commit_message>
feat: standardize specific project tasks to Du An Mau across tasks data, DataModel, Web dashboard and PDF report
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Gauge Chart tiến độ 7 dự án mẫu</t>
+          <t>Gauge Chart tiến độ Dự Án Mẫu</t>
         </is>
       </c>
     </row>
@@ -1223,12 +1223,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Quản lý thiết kế các dự án thuê ngoài chuẩn hóa theo yêu cầu nội bộ</t>
+          <t>Quản lý chuẩn hóa hồ sơ thiết kế chuyển đổi sang mô hình BIM nội bộ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tỷ lệ dự án thuê ngoài tuân thủ chuẩn nội bộ</t>
+          <t>Tỷ lệ dự án thiết kế tuân thủ chuẩn BIM nội bộ</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1416,7 +1416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Quản lý chung</t>
+          <t>Quản lý điều hành</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TBP BIM - Thiết kế</t>
+          <t>Trưởng bộ phận BIM - Thiết kế</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1534,34 +1534,34 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GRP_BIM_XD</t>
+          <t>GRP_TK_BIM_KC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BIM Xây dựng (KT - KC)</t>
+          <t>Thiết kế &amp; BIM Kết cấu</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Trưởng nhóm BIM XD</t>
+          <t>Lead Bộ môn Kết cấu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Nhân sự D (Lead Kết Cấu)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Lead Bộ Môn</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -1584,22 +1584,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GRP_BIM_XD</t>
+          <t>GRP_TK_BIM_KC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BIM Xây dựng (KT - KC)</t>
+          <t>Thiết kế &amp; BIM Kết cấu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kỹ sư BIM KT - KC</t>
+          <t>Kỹ sư TK Kết cấu &amp; Kỹ sư BIM KC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nhân sự H, Nhân sự I, Nhân sự J, Nhân sự K...</t>
+          <t>KS Triển khai KC &amp; 3 KS BIM KC (Nhân sự J, K...)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1608,53 +1608,53 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G4" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Đã chia đều 3 KS BIM về bộ môn</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Biến động T04/2026 &amp; Cần tuyển thêm</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>10</v>
-      </c>
-      <c r="K4" t="n">
-        <v>4</v>
-      </c>
       <c r="L4" t="n">
-        <v>0.7143</v>
+        <v>0.8333</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GRP_BIM_MEPF</t>
+          <t>GRP_TK_BIM_KT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BIM MEPF</t>
+          <t>Thiết kế &amp; BIM Kiến trúc</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Trưởng nhóm BIM MEPF</t>
+          <t>Lead Bộ môn Kiến trúc</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Nhân sự E</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Leader</t>
+          <t>Lead Bộ Môn</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1684,22 +1684,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GRP_BIM_MEPF</t>
+          <t>GRP_TK_BIM_KT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BIM MEPF</t>
+          <t>Thiết kế &amp; BIM Kiến trúc</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kỹ sư BIM MEPF</t>
+          <t>KTS Triển khai &amp; Kỹ sư BIM Kiến trúc</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nhân sự L &amp; KS BIM MEPF</t>
+          <t>KTS Triển khai &amp; 3 KS BIM KT (Nhân sự H, I...)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1708,121 +1708,121 @@
         </is>
       </c>
       <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Đã chia đều 3 KS BIM về bộ môn</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" t="n">
         <v>2</v>
       </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Đang làm việc</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GRP_BIM_HT</t>
+          <t>GRP_TK_BIM_MEP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BIM Hạ tầng</t>
+          <t>Thiết kế &amp; BIM Cơ điện (MEPF)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kỹ sư BIM Hạ tầng</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Nhân sự C (Lead BIM MEPF)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Nhân viên</t>
+          <t>Lead Bộ Môn</t>
         </is>
       </c>
       <c r="F7" t="n">
         <v>2</v>
       </c>
       <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Đang làm việc</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
         <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Đang làm việc</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>2</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GRP_TK_KT</t>
+          <t>GRP_TK_BIM_MEP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Thiết kế Kiến trúc</t>
+          <t>Thiết kế &amp; BIM Cơ điện (MEPF)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chủ trì TK Kiến trúc</t>
+          <t>Kỹ sư TK Cơ Điện &amp; Kỹ sư BIM MEP</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>KS Cơ Điện &amp; 3 KS BIM MEP (Nhân sự L &amp; KS MEP)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Chủ trì</t>
+          <t>Nhân viên</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Đã đủ chủ trì</t>
+          <t>Đã chia đều 3 KS BIM về bộ môn</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -1834,27 +1834,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GRP_TK_KT</t>
+          <t>GRP_TK_BIM_HVAC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Thiết kế Kiến trúc</t>
+          <t>Thiết kế &amp; BIM HVAC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kiến trúc sư triển khai</t>
+          <t>Lead Bộ môn HVAC</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KTS Triển khai</t>
+          <t>Nhân sự G</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Nhân viên</t>
+          <t>Lead Bộ Môn</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1884,31 +1884,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GRP_TK_KC</t>
+          <t>GRP_TK_BIM_HVAC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Thiết kế Kết cấu</t>
+          <t>Thiết kế &amp; BIM HVAC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Chủ trì TK Kết cấu</t>
+          <t>Kỹ sư TK HVAC &amp; Triển khai</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>KS Triển khai HVAC</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Chủ trì</t>
+          <t>Nhân viên</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
@@ -1918,50 +1918,50 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Đã đủ chủ trì</t>
+          <t>Đang làm việc</t>
         </is>
       </c>
       <c r="J10" t="n">
         <v>1</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GRP_TK_KC</t>
+          <t>GRP_BIM_HT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Thiết kế Kết cấu</t>
+          <t>BIM Hạ tầng &amp; CDE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kỹ sư TK Kết cấu</t>
+          <t>Lead BIM Hạ tầng &amp; Quản trị CDE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KS Triển khai KC</t>
+          <t>Nhân sự M</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Nhân viên</t>
+          <t>Lead Bộ Môn</t>
         </is>
       </c>
       <c r="F11" t="n">
         <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1972,213 +1972,63 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GRP_TK_ME</t>
+          <t>GRP_BIM_HT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Thiết kế Điện - Cơ (CTN, PCCC)</t>
+          <t>BIM Hạ tầng &amp; CDE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Chủ trì TK Điện - Cơ</t>
+          <t>Kỹ sư BIM Hạ tầng &amp; CDE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>2 KS BIM Hạ tầng &amp; CDE (Điều phối chia đều sang)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Chủ trì</t>
+          <t>Nhân viên</t>
         </is>
       </c>
       <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" t="n">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Đã chia đều 2 KS BIM về bộ môn</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Đã đủ chủ trì</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
       <c r="L12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>GRP_TK_ME</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Thiết kế Điện - Cơ (CTN, PCCC)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Kỹ sư TK Cơ - Điện</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>KS Triển khai Cơ - Điện</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Nhân viên</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Đang làm việc</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>GRP_TK_HVAC</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Thiết kế HVAC</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Chủ trì TK HVAC</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Nhân sự G</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Chủ trì</t>
-        </is>
-      </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Đã đủ chủ trì</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>GRP_TK_HVAC</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Thiết kế HVAC</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Kỹ sư TK HVAC</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>KS Triển khai HVAC</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Nhân viên</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Đang làm việc</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>1</v>
+        <v>0.6667</v>
       </c>
     </row>
   </sheetData>
@@ -19071,7 +18921,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ChuTriPhuTrach</t>
+          <t>LeadPhuTrach</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -30715,17 +30565,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm nước thải2.1a-BP16.1a (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm xử lý nước thải (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -30767,17 +30617,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng trạm nước thải 2.1a-BP16.1a</t>
+          <t>Triển khai bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -30819,17 +30669,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm nước thải 2.1a-BP16.1a</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -30871,17 +30721,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ BTCT nền trạm nước thải 2.1a-BP16.1a</t>
+          <t>Triển khai bản vẽ BTCT nền trạm xử lý nước thải (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -30923,17 +30773,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ nền trạm nước thải 2.1a-BP16.1a</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ nền trạm xử lý nước thải (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -30975,17 +30825,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm trạm nước thải 2.1a-BP16.1a, tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm trạm xử lý nước thải (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -31027,17 +30877,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bản vẽ vách bể BP15.2 lần 1</t>
+          <t>Thực hiện điều chỉnh bản vẽ vách bể kỹ thuật (Dự Án Mẫu) lần 1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -31079,17 +30929,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Triển khai bảng khối lượng cốt thép vách bể BP15.2</t>
+          <t>Triển khai bảng khối lượng cốt thép vách bể kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -31131,17 +30981,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần vách bể  2.1a-BP16.1a, tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần vách bể trạm xử lý nước thải (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -31183,17 +31033,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà xỉ than BP12  (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà phụ trợ kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -31235,17 +31085,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng nhà xỉ than BP12</t>
+          <t>Triển khai bản vẽ đà kiềng nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -31287,17 +31137,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà xỉ than BP12</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -31339,17 +31189,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà xỉ than BP12, tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà phụ trợ kỹ thuật (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -31391,17 +31241,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm nước thải BP15.1  (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm xử lý nước thải (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -31443,17 +31293,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng trạm nước thải BP15.1</t>
+          <t>Triển khai bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -31495,17 +31345,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm nước thải BP15.1</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -31547,17 +31397,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà nồi hơi BP12</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà nồi hơi kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -31599,17 +31449,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng nhà nồi hơi BP12</t>
+          <t>Triển khai bản vẽ đà kiềng nhà nồi hơi kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -31651,17 +31501,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà nồi hơi BP12</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà nồi hơi kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -31703,17 +31553,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà nồi hơi BP12, tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà nồi hơi kỹ thuật (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -31755,17 +31605,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục  BP3 lần 1</t>
+          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục mái xưởng A (Dự Án Mẫu) lần 1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -31807,17 +31657,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục  MS1 lần 1</t>
+          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục xưởng sản xuất (Dự Án Mẫu) lần 1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -31859,17 +31709,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép hạng mục MS1 cùng nhà thầu Fuji</t>
+          <t>Kiểm soát thiết kế kết cấu thép hạng mục xưởng sản xuất (Dự Án Mẫu) cùng Đơn vị gia công kết cấu thép</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -31907,17 +31757,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép hạng mục BP3, BP12 cùng nhà thầu CPT</t>
+          <t>Kiểm soát thiết kế kết cấu thép các hạng mục kết cấu thép Dự Án Mẫu cùng Đơn vị gia công kết cấu thép</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -31951,17 +31801,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần mái phục vụ phối hợp va chạm NP42</t>
+          <t>Triển khai mô hình 3D phần mái phục vụ phối hợp va chạm khu nhà điều hành (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -32003,17 +31853,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ BTCT sàn mái NP42</t>
+          <t>Triển khai bản vẽ BTCT sàn mái khu nhà điều hành (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -32055,17 +31905,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ BTCT sàn mái NP42</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ BTCT sàn mái khu nhà điều hành (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -32107,12 +31957,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -32159,17 +32009,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ BTCT dầm mái NP42</t>
+          <t>Triển khai bản vẽ BTCT dầm mái khu nhà điều hành (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -32211,17 +32061,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ dầm BTCT tầng mái NP42</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ dầm BTCT tầng mái khu nhà điều hành (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -32263,17 +32113,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bộ bản vẽ dầm tầng mái TH2 lần 1</t>
+          <t>Thực hiện điều chỉnh bộ bản vẽ dầm tầng mái khu nhà xưởng B (Dự Án Mẫu) lần 1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -32315,17 +32165,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bộ bản vẽ thang bộ  tầng mái TH1 lần 2</t>
+          <t>Thực hiện điều chỉnh bộ bản vẽ thang bộ tầng mái khu nhà xưởng A (Dự Án Mẫu) lần 2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -32367,17 +32217,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Thực hiện mô hình 3D tường xây TH2 (bao gồm lanh tô, bổ trụ, giằng tường, cửa) để phối hợp va chạm</t>
+          <t>Thực hiện mô hình 3D tường xây khu nhà xưởng B (Dự Án Mẫu) (bao gồm lanh tô, bổ trụ, giằng tường, cửa) để phối hợp va chạm</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -32419,17 +32269,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop xây tô  tầng 1 TH2</t>
+          <t>Triển khai bản vẽ Shop xây tô tầng 1 khu nhà xưởng B (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -32471,12 +32321,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -32523,12 +32373,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -32575,12 +32425,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -32627,12 +32477,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -32679,12 +32529,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -32731,12 +32581,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -32783,12 +32633,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -32831,17 +32681,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Phối hợp soạn và cấp thông tin khối lương, mô hình, bản vẽ phục vụ IPC</t>
+          <t>Phối hợp soạn và cấp thông tin khối lương, mô hình, bản vẽ phục vụ hồ sơ nghiệm thu IPC (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -32875,12 +32725,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -32927,17 +32777,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát nhà văn phòng các xưởng</t>
+          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát khu văn phòng (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -32975,17 +32825,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng gạch ốp lát văn phòng các xưởng</t>
+          <t>Triển khai các bảng khối lượng gạch ốp lát khu văn phòng (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -33027,17 +32877,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D ốp lát hoàn thiện nhà vệ sinh 1,2</t>
+          <t>Triển khai mô hình 3D ốp lát hoàn thiện khu vệ sinh (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -33079,17 +32929,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát nhà vệ sinh 1,2</t>
+          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát khu vệ sinh (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -33127,17 +32977,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng gạch ốp lát nhà vệ sinh 1,2</t>
+          <t>Triển khai các bảng khối lượng gạch ốp lát khu vệ sinh (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -33179,17 +33029,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D ốp lát hoàn thiện nhà  bảo vệ 1,2</t>
+          <t>Triển khai mô hình 3D ốp lát hoàn thiện nhà bảo vệ (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -33231,17 +33081,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát nhà bảo vệ 1,2</t>
+          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát nhà bảo vệ (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -33279,17 +33129,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng gạch ốp lát nhà bảo vệ 1,2</t>
+          <t>Triển khai các bảng khối lượng gạch ốp lát nhà bảo vệ (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -33331,12 +33181,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -33379,12 +33229,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -33431,17 +33281,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Điều chỉnh và phát hành mô hình 3D cho tất cả các thay đổi thiết kế dự án</t>
+          <t>Điều chỉnh và phát hành mô hình 3D cho tất cả các thay đổi thiết kế Dự Án Mẫu</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -33483,17 +33333,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần  phục vụ phối hợp va chạm nhà phụ trợ 1 (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần phục vụ phối hợp va chạm nhà phụ trợ kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -33535,17 +33385,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop đà kiềng và nền bể chứa và bể XLNT nhà phụ trợ 1</t>
+          <t>Triển khai bản vẽ Shop đà kiềng và nền bể chứa và bể XLNT nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -33587,17 +33437,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng và nền nhà phụ trợ 1</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng và nền nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -33631,12 +33481,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -33683,12 +33533,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -33735,12 +33585,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -33787,12 +33637,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -33835,12 +33685,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -33879,12 +33729,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -33923,12 +33773,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -33967,12 +33817,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -34011,12 +33861,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -34055,17 +33905,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Triển  khai các bảng khối lương hệ thống điện hạ tầng</t>
+          <t>Triển khai các bảng khối lương hệ thống điện hạ tầng</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -34099,17 +33949,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép nhà xưởng E, G, H</t>
+          <t>Kiểm soát thiết kế kết cấu thép cụm nhà xưởng mở rộng (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -34143,17 +33993,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép các xưởng A, B, C, D, F cùng nhà thầu Đại Dũng</t>
+          <t>Kiểm soát thiết kế kết cấu thép cụm nhà xưởng sản xuất chính (Dự Án Mẫu) cùng Đơn vị gia công kết cấu thép</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -34187,17 +34037,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Triẻn khai mô hình 3D phục vụ phối hợp va chạm phần ngầm bể tự hoại  (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý) (tách 2 gói)</t>
+          <t>Triẻn khai mô hình 3D phục vụ phối hợp va chạm phần ngầm bể tự hoại (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý) (tách 2 gói)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -34239,12 +34089,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -34291,12 +34141,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -34343,12 +34193,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -34395,17 +34245,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột 2 gói 3.2B và 3.2C theo yêu cầu BCH (tách gói, chạy tọa độ)</t>
+          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột các phân đoạn móng (Dự Án Mẫu) theo yêu cầu BCH (tách gói, chạy tọa độ)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -34447,17 +34297,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép móng và cổ cột cho 3.2B và 3.2C</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép móng và cổ cột cho các phân đoạn móng (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -34499,12 +34349,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -34551,17 +34401,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột 2 gói 3.2B và 3.2C theo comments TVGS lần 1</t>
+          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột các phân đoạn móng (Dự Án Mẫu) theo comments TVGS lần 1</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -34599,12 +34449,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -34647,17 +34497,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D xây tô hà trạm 1,2,3,4 (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D xây tô nhà trạm kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -34699,17 +34549,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ shop xây tô nhà trạm 1,2,3,4</t>
+          <t>Triển khai bản vẽ shop xây tô nhà trạm kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -34751,17 +34601,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng xây tô nhà trạm 1,2,3,4</t>
+          <t>Triển khai các bảng khối lượng xây tô nhà trạm kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -34803,17 +34653,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D ốp lát nhà vệ sinh trạm nguồn 1,2,3,4 (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D ốp lát nhà vệ sinh trạm nguồn điện kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -34855,17 +34705,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ shop ốp lát nhà vệ sinh trạm nguồn 1,2,3,4</t>
+          <t>Triển khai bản vẽ shop ốp lát nhà vệ sinh trạm nguồn điện kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -34907,17 +34757,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng ốp lát nhà trạm nguồn 1,2,3,4</t>
+          <t>Triển khai các bảng khối lượng ốp lát trạm nguồn điện kỹ thuật (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -34959,17 +34809,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Triển khai bảng khối lượng chi tiết trạm nguồn phục vụ triển khai IPC1</t>
+          <t>Triển khai bảng khối lượng chi tiết trạm nguồn điện kỹ thuật (Dự Án Mẫu) phục vụ hồ sơ nghiệm thu IPC (Dự Án Mẫu)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -35011,12 +34861,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -35063,12 +34913,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Dự án Mẫu (Thi công &amp; Triển khai)</t>
+          <t>Quản trị &amp; Tổ chức</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Dự án Mẫu</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -36165,7 +36015,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Chuẩn hoá thiết kế kiến trúc  các hạng mục</t>
+          <t>Chuẩn hoá thiết kế kiến trúc các hạng mục</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -38981,7 +38831,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Biểu mẫu câu hỏi làm rõ thông tin kĩ thuật  đầu vào khi triển khai dự án</t>
+          <t>Biểu mẫu câu hỏi làm rõ thông tin kĩ thuật đầu vào khi triển khai dự án</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
@@ -39773,7 +39623,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Biểu mẫu câu hỏi làm rõ thông tin kĩ thuật  đầu vào khi triển khai dự án</t>
+          <t>Biểu mẫu câu hỏi làm rõ thông tin kĩ thuật đầu vào khi triển khai dự án</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">

</xml_diff>

<commit_message>
feat: separate 87 tasks into 7 distinct Du An Mau (01 to 07) across dashboard, excel and pdf report
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -30570,12 +30570,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm xử lý nước thải (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm xử lý nước thải (Dự Án Mẫu 02) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -30622,12 +30622,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -30674,12 +30674,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -30726,12 +30726,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ BTCT nền trạm xử lý nước thải (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ BTCT nền trạm xử lý nước thải (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -30778,12 +30778,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ nền trạm xử lý nước thải (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ nền trạm xử lý nước thải (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -30830,12 +30830,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm trạm xử lý nước thải (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm trạm xử lý nước thải (Dự Án Mẫu 02), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -30882,12 +30882,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bản vẽ vách bể kỹ thuật (Dự Án Mẫu) lần 1</t>
+          <t>Thực hiện điều chỉnh bản vẽ vách bể kỹ thuật (Dự Án Mẫu 02) lần 1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -30934,12 +30934,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Triển khai bảng khối lượng cốt thép vách bể kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai bảng khối lượng cốt thép vách bể kỹ thuật (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -30986,12 +30986,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần vách bể trạm xử lý nước thải (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần vách bể trạm xử lý nước thải (Dự Án Mẫu 02), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -31038,12 +31038,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà phụ trợ kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà phụ trợ kỹ thuật (Dự Án Mẫu 02) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -31090,12 +31090,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ đà kiềng nhà phụ trợ kỹ thuật (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -31142,12 +31142,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà phụ trợ kỹ thuật (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -31194,12 +31194,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà phụ trợ kỹ thuật (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà phụ trợ kỹ thuật (Dự Án Mẫu 02), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -31246,12 +31246,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm xử lý nước thải (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm trạm xử lý nước thải (Dự Án Mẫu 02) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -31298,12 +31298,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -31350,12 +31350,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng trạm xử lý nước thải (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -31402,12 +31402,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà nồi hơi kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai mô hình 3D phần ngầm phục vụ phối hợp va chạm nhà nồi hơi kỹ thuật (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -31454,12 +31454,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ đà kiềng nhà nồi hơi kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ đà kiềng nhà nồi hơi kỹ thuật (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -31506,12 +31506,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà nồi hơi kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng nhà nồi hơi kỹ thuật (Dự Án Mẫu 02)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -31558,12 +31558,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà nồi hơi kỹ thuật (Dự Án Mẫu), tập hợp soạn RFI nếu cần</t>
+          <t>Trao đổi làm rõ thiếu xót thông tin thiết kế phần ngầm nhà nồi hơi kỹ thuật (Dự Án Mẫu 02), tập hợp soạn RFI nếu cần</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -31610,12 +31610,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục mái xưởng A (Dự Án Mẫu) lần 1</t>
+          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục mái xưởng A (Dự Án Mẫu 03) lần 1</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -31662,12 +31662,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục xưởng sản xuất (Dự Án Mẫu) lần 1</t>
+          <t>Thực hiện điều chỉnh mô hình và bản vẽ Shop thoát nước mưa mái hạng mục xưởng sản xuất (Dự Án Mẫu 03) lần 1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -31714,12 +31714,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép hạng mục xưởng sản xuất (Dự Án Mẫu) cùng Đơn vị gia công kết cấu thép</t>
+          <t>Kiểm soát thiết kế kết cấu thép hạng mục xưởng sản xuất (Dự Án Mẫu 03) cùng Đơn vị gia công kết cấu thép</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -31762,12 +31762,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 01</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép các hạng mục kết cấu thép Dự Án Mẫu cùng Đơn vị gia công kết cấu thép</t>
+          <t>Kiểm soát thiết kế kết cấu thép các hạng mục kết cấu thép (Dự Án Mẫu 03) cùng Đơn vị gia công kết cấu thép</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -31806,12 +31806,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần mái phục vụ phối hợp va chạm khu nhà điều hành (Dự Án Mẫu)</t>
+          <t>Triển khai mô hình 3D phần mái phục vụ phối hợp va chạm khu nhà điều hành (Dự Án Mẫu 03)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -31858,12 +31858,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ BTCT sàn mái khu nhà điều hành (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ BTCT sàn mái khu nhà điều hành (Dự Án Mẫu 03)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -31910,12 +31910,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ BTCT sàn mái khu nhà điều hành (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ BTCT sàn mái khu nhà điều hành (Dự Án Mẫu 03)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -31962,7 +31962,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -32014,12 +32014,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ BTCT dầm mái khu nhà điều hành (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ BTCT dầm mái khu nhà điều hành (Dự Án Mẫu 03)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -32066,12 +32066,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ dầm BTCT tầng mái khu nhà điều hành (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ dầm BTCT tầng mái khu nhà điều hành (Dự Án Mẫu 03)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -32118,12 +32118,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bộ bản vẽ dầm tầng mái khu nhà xưởng B (Dự Án Mẫu) lần 1</t>
+          <t>Thực hiện điều chỉnh bộ bản vẽ dầm tầng mái khu nhà xưởng B (Dự Án Mẫu 04) lần 1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -32170,12 +32170,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bộ bản vẽ thang bộ tầng mái khu nhà xưởng A (Dự Án Mẫu) lần 2</t>
+          <t>Thực hiện điều chỉnh bộ bản vẽ thang bộ tầng mái khu nhà xưởng A (Dự Án Mẫu 04) lần 2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -32222,12 +32222,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Thực hiện mô hình 3D tường xây khu nhà xưởng B (Dự Án Mẫu) (bao gồm lanh tô, bổ trụ, giằng tường, cửa) để phối hợp va chạm</t>
+          <t>Thực hiện mô hình 3D tường xây khu nhà xưởng B (Dự Án Mẫu 04) (bao gồm lanh tô, bổ trụ, giằng tường, cửa) để phối hợp va chạm</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -32274,12 +32274,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop xây tô tầng 1 khu nhà xưởng B (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ Shop xây tô tầng 1 khu nhà xưởng B (Dự Án Mẫu 04)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -32326,7 +32326,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -32378,7 +32378,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 04</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -32430,7 +32430,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -32482,7 +32482,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -32534,7 +32534,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -32586,7 +32586,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -32638,7 +32638,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -32686,12 +32686,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Phối hợp soạn và cấp thông tin khối lương, mô hình, bản vẽ phục vụ hồ sơ nghiệm thu IPC (Dự Án Mẫu)</t>
+          <t>Phối hợp soạn và cấp thông tin khối lương, mô hình, bản vẽ phục vụ hồ sơ nghiệm thu IPC (Dự Án Mẫu 05)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -32730,7 +32730,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -32782,12 +32782,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát khu văn phòng (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát khu văn phòng xưởng (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -32830,12 +32830,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng gạch ốp lát khu văn phòng (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng gạch ốp lát khu văn phòng xưởng (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -32882,12 +32882,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D ốp lát hoàn thiện khu vệ sinh (Dự Án Mẫu)</t>
+          <t>Triển khai mô hình 3D ốp lát hoàn thiện khu vệ sinh (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -32934,12 +32934,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát khu vệ sinh (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát khu vệ sinh (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -32982,12 +32982,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng gạch ốp lát khu vệ sinh (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng gạch ốp lát khu vệ sinh (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -33034,12 +33034,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D ốp lát hoàn thiện nhà bảo vệ (Dự Án Mẫu)</t>
+          <t>Triển khai mô hình 3D ốp lát hoàn thiện nhà bảo vệ (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -33086,12 +33086,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát nhà bảo vệ (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ Shop hoàn thiện ốp lát nhà bảo vệ (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -33134,12 +33134,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng gạch ốp lát nhà bảo vệ (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng gạch ốp lát nhà bảo vệ (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -33186,7 +33186,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -33234,7 +33234,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -33286,12 +33286,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 02</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Điều chỉnh và phát hành mô hình 3D cho tất cả các thay đổi thiết kế Dự Án Mẫu</t>
+          <t>Điều chỉnh và phát hành mô hình 3D cho tất cả các thay đổi thiết kế dự án mẫu</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -33338,12 +33338,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D phần phục vụ phối hợp va chạm nhà phụ trợ kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D phần phục vụ phối hợp va chạm nhà phụ trợ kỹ thuật (Dự Án Mẫu 01) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -33390,12 +33390,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ Shop đà kiềng và nền bể chứa và bể XLNT nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ Shop đà kiềng và nền bể chứa và bể XLNT nhà phụ trợ kỹ thuật (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -33442,12 +33442,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng và nền nhà phụ trợ kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép, ván khuôn và các khối lượng xuất từ bản vẽ đà kiềng và nền nhà phụ trợ kỹ thuật (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -33486,7 +33486,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -33538,7 +33538,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -33590,7 +33590,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -33642,7 +33642,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -33690,7 +33690,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -33734,7 +33734,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -33778,7 +33778,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -33822,7 +33822,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -33866,7 +33866,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -33910,7 +33910,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -33954,12 +33954,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép cụm nhà xưởng mở rộng (Dự Án Mẫu)</t>
+          <t>Kiểm soát thiết kế kết cấu thép cụm nhà xưởng mở rộng (Dự Án Mẫu 01)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -33998,12 +33998,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 03</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Kiểm soát thiết kế kết cấu thép cụm nhà xưởng sản xuất chính (Dự Án Mẫu) cùng Đơn vị gia công kết cấu thép</t>
+          <t>Kiểm soát thiết kế kết cấu thép cụm nhà xưởng sản xuất chính (Dự Án Mẫu 01) cùng Đơn vị gia công kết cấu thép</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -34042,7 +34042,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -34094,7 +34094,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -34146,7 +34146,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -34198,7 +34198,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -34250,12 +34250,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột các phân đoạn móng (Dự Án Mẫu) theo yêu cầu BCH (tách gói, chạy tọa độ)</t>
+          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột các phân đoạn móng (Dự Án Mẫu 07) theo yêu cầu BCH (tách gói, chạy tọa độ)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -34302,12 +34302,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng bê tông, cốt thép móng và cổ cột cho các phân đoạn móng (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng bê tông, cốt thép móng và cổ cột cho các phân đoạn móng (Dự Án Mẫu 07)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -34354,7 +34354,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -34406,12 +34406,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột các phân đoạn móng (Dự Án Mẫu) theo comments TVGS lần 1</t>
+          <t>Thực hiện điều chỉnh bản vẽ Shop móng và cổ cột các phân đoạn móng (Dự Án Mẫu 07) theo comments TVGS lần 1</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -34454,7 +34454,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 05</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -34502,12 +34502,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D xây tô nhà trạm kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D xây tô nhà trạm kỹ thuật (Dự Án Mẫu 06) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -34554,12 +34554,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ shop xây tô nhà trạm kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ shop xây tô nhà trạm kỹ thuật (Dự Án Mẫu 06)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -34606,12 +34606,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng xây tô nhà trạm kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng xây tô nhà trạm kỹ thuật (Dự Án Mẫu 06)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -34658,12 +34658,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Triển khai mô hình 3D ốp lát nhà vệ sinh trạm nguồn điện kỹ thuật (Dự Án Mẫu) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
+          <t>Triển khai mô hình 3D ốp lát nhà vệ sinh trạm nguồn điện kỹ thuật (Dự Án Mẫu 06) (phát hiện lỗi, báo cáo, đề xuất phương án, trao đổi các bên xử lý)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -34710,12 +34710,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Triển khai bản vẽ shop ốp lát nhà vệ sinh trạm nguồn điện kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai bản vẽ shop ốp lát nhà vệ sinh trạm nguồn điện kỹ thuật (Dự Án Mẫu 06)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -34762,12 +34762,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Triển khai các bảng khối lượng ốp lát trạm nguồn điện kỹ thuật (Dự Án Mẫu)</t>
+          <t>Triển khai các bảng khối lượng ốp lát trạm nguồn điện kỹ thuật (Dự Án Mẫu 06)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -34814,12 +34814,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 06</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Triển khai bảng khối lượng chi tiết trạm nguồn điện kỹ thuật (Dự Án Mẫu) phục vụ hồ sơ nghiệm thu IPC (Dự Án Mẫu)</t>
+          <t>Triển khai bảng khối lượng chi tiết trạm nguồn điện kỹ thuật (Dự Án Mẫu 06) phục vụ hồ sơ nghiệm thu IPC (Dự Án Mẫu 05)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -34866,7 +34866,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 07</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -34918,7 +34918,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu</t>
+          <t>Dự Án Mẫu 07</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">

</xml_diff>

<commit_message>
feat: refine strategy report with role-based HR, agile SLA (Shop 5d/Combine 3d/QS 3d), AI Agent automation and parallel pilot project
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -1499,7 +1499,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nhân sự D (Lead Kết Cấu)</t>
+          <t>Lead Bộ môn Kết cấu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KS Triển khai KC &amp; 3 KS BIM KC (Nhân sự J, K...)</t>
+          <t>2 KS Thiết kế &amp; 3 KS BIM Kết cấu</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Bộ môn Kiến trúc</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KTS Triển khai &amp; 3 KS BIM KT (Nhân sự H, I...)</t>
+          <t>1 KTS Thiết kế &amp; 3 KS BIM Kiến trúc</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Nhân sự C (Lead BIM MEPF)</t>
+          <t>Lead Bộ môn BIM MEPF</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KS Cơ Điện &amp; 3 KS BIM MEP (Nhân sự L &amp; KS MEP)</t>
+          <t>1 KS TK + 1 KS MEP + 3 KS BIM MEP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead Bộ môn HVAC</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KS Triển khai HVAC</t>
+          <t>1 KS Triển khai HVAC</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Lead Kỹ thuật Hạ tầng &amp; CDE</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2 KS BIM Hạ tầng &amp; CDE (Điều phối chia đều sang)</t>
+          <t>2 KS BIM Hạ tầng &amp; CDE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2593,12 +2593,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3217,7 +3217,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3321,7 +3321,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -3529,12 +3529,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3737,7 +3737,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3997,12 +3997,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -4257,7 +4257,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -4465,12 +4465,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4621,7 +4621,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4777,7 +4777,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4933,12 +4933,12 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -5297,7 +5297,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5401,12 +5401,12 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5453,7 +5453,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -5505,7 +5505,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -5557,7 +5557,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -5609,7 +5609,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -5869,12 +5869,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -5921,7 +5921,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -6181,7 +6181,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -6285,7 +6285,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -6337,12 +6337,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -6441,7 +6441,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -6493,7 +6493,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -6545,7 +6545,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -6597,7 +6597,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -6649,7 +6649,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -6805,12 +6805,12 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -6909,7 +6909,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -6961,7 +6961,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -7013,7 +7013,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -7117,7 +7117,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -7221,7 +7221,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -7273,12 +7273,12 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -7325,7 +7325,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -7429,7 +7429,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -7481,7 +7481,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -7585,7 +7585,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -7689,7 +7689,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -7741,12 +7741,12 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -7793,7 +7793,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -7949,7 +7949,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -8053,7 +8053,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -8209,12 +8209,12 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -8313,7 +8313,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -8365,7 +8365,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -8417,7 +8417,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -8469,7 +8469,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -8573,7 +8573,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -8625,7 +8625,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -8677,12 +8677,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -8729,7 +8729,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -8833,7 +8833,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -8885,7 +8885,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -8937,7 +8937,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -8989,7 +8989,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -9041,7 +9041,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -9145,12 +9145,12 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -9197,7 +9197,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -9301,7 +9301,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -9353,7 +9353,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -9405,7 +9405,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -9457,7 +9457,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -9509,7 +9509,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -9613,12 +9613,12 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -9665,7 +9665,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -9717,7 +9717,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -9769,7 +9769,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -9821,7 +9821,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -9925,7 +9925,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -9977,7 +9977,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -10081,12 +10081,12 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -10133,7 +10133,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -10185,7 +10185,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -10237,7 +10237,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -10289,7 +10289,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -10393,7 +10393,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -10445,7 +10445,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -10549,12 +10549,12 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -10705,7 +10705,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -10757,7 +10757,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -10861,7 +10861,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -10913,7 +10913,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -11017,12 +11017,12 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -11069,7 +11069,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -11225,7 +11225,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -11329,7 +11329,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -11381,7 +11381,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -11485,12 +11485,12 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -11537,7 +11537,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -11589,7 +11589,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -11641,7 +11641,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -11797,7 +11797,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -11849,7 +11849,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -11953,12 +11953,12 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -12109,7 +12109,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -12161,7 +12161,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -12213,7 +12213,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -12265,7 +12265,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -12317,7 +12317,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -12369,7 +12369,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -12421,12 +12421,12 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -12577,7 +12577,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -12681,7 +12681,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -12733,7 +12733,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -12837,7 +12837,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -12889,12 +12889,12 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -12941,7 +12941,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -12993,7 +12993,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -13097,7 +13097,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -13201,7 +13201,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -13253,7 +13253,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -13305,7 +13305,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -13357,12 +13357,12 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -13409,7 +13409,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -13513,7 +13513,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -13565,7 +13565,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -13617,7 +13617,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -13669,7 +13669,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -13721,7 +13721,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -13773,7 +13773,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -13825,12 +13825,12 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -13981,7 +13981,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -14033,7 +14033,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -14085,7 +14085,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -14137,7 +14137,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -14189,7 +14189,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -14241,7 +14241,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -14293,12 +14293,12 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -14345,7 +14345,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -14397,7 +14397,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -14501,7 +14501,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -14553,7 +14553,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -14605,7 +14605,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -14657,7 +14657,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -14761,12 +14761,12 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -14813,7 +14813,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -14865,7 +14865,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -14917,7 +14917,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -14969,7 +14969,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -15021,7 +15021,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -15073,7 +15073,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -15177,7 +15177,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -15229,12 +15229,12 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
@@ -15281,7 +15281,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -15333,7 +15333,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -15385,7 +15385,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -15437,7 +15437,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -15489,7 +15489,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -15541,7 +15541,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -15593,7 +15593,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -15645,7 +15645,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -15697,12 +15697,12 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -15749,7 +15749,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -15853,7 +15853,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -15905,7 +15905,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
@@ -15957,7 +15957,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -16009,7 +16009,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -16113,7 +16113,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -16165,12 +16165,12 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -16217,7 +16217,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
@@ -16269,7 +16269,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -16321,7 +16321,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -16373,7 +16373,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -16477,7 +16477,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -16529,7 +16529,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -16581,7 +16581,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -16633,12 +16633,12 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H281" t="inlineStr">
@@ -16685,7 +16685,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -16737,7 +16737,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -16789,7 +16789,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -16841,7 +16841,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -16893,7 +16893,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -16945,7 +16945,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -16997,7 +16997,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -17049,7 +17049,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -17101,12 +17101,12 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
@@ -17153,7 +17153,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -17205,7 +17205,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -17257,7 +17257,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -17309,7 +17309,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -17361,7 +17361,7 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -17413,7 +17413,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
@@ -17465,7 +17465,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -17569,12 +17569,12 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>Nhân sự A</t>
+          <t>Trưởng bộ phận BIM - TK</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>TBP BIM-TK</t>
+          <t>Ban Quản lý</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
@@ -17621,7 +17621,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Nhân sự B</t>
+          <t>Lead BIM Kiến Trúc</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
@@ -17673,7 +17673,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>Nhân sự H</t>
+          <t>Kỹ sư BIM Kiến Trúc 1</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
@@ -17725,7 +17725,7 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>Nhân sự I</t>
+          <t>Kỹ sư BIM Kiến Trúc 2</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
@@ -17777,7 +17777,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>Nhân sự J</t>
+          <t>Kỹ sư BIM Kết Cấu 1</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
@@ -17829,7 +17829,7 @@
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>Nhân sự K</t>
+          <t>Kỹ sư BIM Kết Cấu 2</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
@@ -17881,7 +17881,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Nhân sự C</t>
+          <t>Lead BIM MEPF</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
@@ -17933,7 +17933,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>Nhân sự L</t>
+          <t>Kỹ sư BIM MEPF</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
@@ -17985,7 +17985,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Nhân sự M</t>
+          <t>Kỹ sư BIM Hạ Tầng &amp; CDE</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -18988,7 +18988,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -19051,7 +19051,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -19114,7 +19114,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -19177,7 +19177,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -19240,7 +19240,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -19303,7 +19303,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -19366,7 +19366,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -19429,7 +19429,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -19492,7 +19492,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -19555,7 +19555,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -19618,7 +19618,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -19681,7 +19681,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -19744,7 +19744,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -19807,7 +19807,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -19870,7 +19870,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -19933,7 +19933,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -20059,7 +20059,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -20122,7 +20122,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -20185,7 +20185,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -20248,7 +20248,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -20374,7 +20374,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Nhân sự D</t>
+          <t>Lead Kết Cấu</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -20437,7 +20437,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -20500,7 +20500,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -20563,7 +20563,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -20626,7 +20626,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -20689,7 +20689,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -20752,7 +20752,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -20815,7 +20815,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -20878,7 +20878,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -20941,7 +20941,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -21004,7 +21004,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -21067,7 +21067,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -21130,7 +21130,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -21193,7 +21193,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -21256,7 +21256,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -21319,7 +21319,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -21382,7 +21382,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -21445,7 +21445,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -21508,7 +21508,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -21571,7 +21571,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -21634,7 +21634,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Nhân sự E</t>
+          <t>Lead Kiến Trúc</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -21697,7 +21697,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -21760,7 +21760,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -21823,7 +21823,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -21886,7 +21886,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -21949,7 +21949,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -22012,7 +22012,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -22075,7 +22075,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -22138,7 +22138,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -22201,7 +22201,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -22264,7 +22264,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -22327,7 +22327,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -22390,7 +22390,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -22453,7 +22453,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -22516,7 +22516,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -22579,7 +22579,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -22642,7 +22642,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -22705,7 +22705,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -22768,7 +22768,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Điện</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -22831,7 +22831,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -22894,7 +22894,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -22957,7 +22957,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -23020,7 +23020,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -23083,7 +23083,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -23146,7 +23146,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -23209,7 +23209,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -23272,7 +23272,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -23335,7 +23335,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -23398,7 +23398,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -23461,7 +23461,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -23524,7 +23524,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -23587,7 +23587,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -23650,7 +23650,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -23713,7 +23713,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -23776,7 +23776,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -23839,7 +23839,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Nhân sự G</t>
+          <t>Lead HVAC</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -23965,7 +23965,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -24028,7 +24028,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -24091,7 +24091,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -24154,7 +24154,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -24217,7 +24217,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -24280,7 +24280,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -24343,7 +24343,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -24406,7 +24406,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -24469,7 +24469,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -24532,7 +24532,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -24595,7 +24595,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -24658,7 +24658,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -24721,7 +24721,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -24784,7 +24784,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -24847,7 +24847,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -24910,7 +24910,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -24973,7 +24973,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -25036,7 +25036,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead Cấp Thoát Nước</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -25099,7 +25099,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E99" t="n">
@@ -25162,7 +25162,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -25225,7 +25225,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -25288,7 +25288,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -25351,7 +25351,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -25414,7 +25414,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -25477,7 +25477,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -25540,7 +25540,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -25603,7 +25603,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -25666,7 +25666,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -25729,7 +25729,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -25792,7 +25792,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -25855,7 +25855,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -25918,7 +25918,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -25981,7 +25981,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -26044,7 +26044,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -26107,7 +26107,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -26170,7 +26170,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Nhân sự F</t>
+          <t>Lead PCCC</t>
         </is>
       </c>
       <c r="E116" t="n">

</xml_diff>

<commit_message>
feat: redesign cover page with full-bleed executive background and standardize project to Du An Mau (removed Mega)
</commit_message>
<xml_diff>
--- a/BIM_TK_PowerBI_DataModel_2026.xlsx
+++ b/BIM_TK_PowerBI_DataModel_2026.xlsx
@@ -30565,12 +30565,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -30617,12 +30617,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -30669,12 +30669,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -30721,12 +30721,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -30773,12 +30773,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -30825,12 +30825,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -30877,12 +30877,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -30929,12 +30929,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -30981,12 +30981,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -31033,12 +31033,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -31085,12 +31085,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -31137,12 +31137,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -31189,12 +31189,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -31241,12 +31241,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -31293,12 +31293,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -31345,12 +31345,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -31397,12 +31397,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -31449,12 +31449,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -31501,12 +31501,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -31553,12 +31553,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -31605,12 +31605,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -31657,12 +31657,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -31709,12 +31709,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -31757,12 +31757,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA (Thực chiến triển khai)</t>
+          <t>Dự Án Mẫu (Thực chiến triển khai)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Dự Án Mẫu MEGA</t>
+          <t>Dự Án Mẫu</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">

</xml_diff>